<commit_message>
Daily Satellite Data Update
</commit_message>
<xml_diff>
--- a/output/HaP_Teplice.xlsx
+++ b/output/HaP_Teplice.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="211">
   <si>
     <t>Datum</t>
   </si>
@@ -70,15 +70,6 @@
     <t>Vysoká</t>
   </si>
   <si>
-    <t>20260822--01</t>
-  </si>
-  <si>
-    <t>20260822--02</t>
-  </si>
-  <si>
-    <t>20260822--03</t>
-  </si>
-  <si>
     <t>20260823--01</t>
   </si>
   <si>
@@ -142,27 +133,30 @@
     <t>20260828--03</t>
   </si>
   <si>
-    <t>05:11</t>
-  </si>
-  <si>
-    <t>04:27</t>
+    <t>20260829--01</t>
+  </si>
+  <si>
+    <t>20260829--02</t>
+  </si>
+  <si>
+    <t>20260829--03</t>
+  </si>
+  <si>
+    <t>05:33</t>
+  </si>
+  <si>
+    <t>03:20</t>
+  </si>
+  <si>
+    <t>05:47</t>
+  </si>
+  <si>
+    <t>03:15</t>
   </si>
   <si>
     <t>05:55</t>
   </si>
   <si>
-    <t>05:33</t>
-  </si>
-  <si>
-    <t>03:21</t>
-  </si>
-  <si>
-    <t>05:47</t>
-  </si>
-  <si>
-    <t>03:15</t>
-  </si>
-  <si>
     <t>04:24</t>
   </si>
   <si>
@@ -202,6 +196,15 @@
     <t>04:15</t>
   </si>
   <si>
+    <t>05:13</t>
+  </si>
+  <si>
+    <t>05:56</t>
+  </si>
+  <si>
+    <t>04:58</t>
+  </si>
+  <si>
     <t>00:00</t>
   </si>
   <si>
@@ -217,13 +220,10 @@
     <t>02:41</t>
   </si>
   <si>
-    <t>01:19:29</t>
-  </si>
-  <si>
-    <t>21:17:00</t>
-  </si>
-  <si>
-    <t>22:53:18</t>
+    <t>04:41</t>
+  </si>
+  <si>
+    <t>01:09</t>
   </si>
   <si>
     <t>00:30:10</t>
@@ -256,7 +256,7 @@
     <t>22:01:58</t>
   </si>
   <si>
-    <t>23:38:55</t>
+    <t>23:38:56</t>
   </si>
   <si>
     <t>19:36:10</t>
@@ -271,7 +271,7 @@
     <t>18:46:54</t>
   </si>
   <si>
-    <t>20:22:57</t>
+    <t>20:22:58</t>
   </si>
   <si>
     <t>21:59:44</t>
@@ -280,7 +280,7 @@
     <t>23:36:55</t>
   </si>
   <si>
-    <t>19:33:24</t>
+    <t>19:33:25</t>
   </si>
   <si>
     <t>21:10:05</t>
@@ -289,13 +289,13 @@
     <t>22:47:08</t>
   </si>
   <si>
-    <t>01:21:54</t>
-  </si>
-  <si>
-    <t>21:19:35</t>
-  </si>
-  <si>
-    <t>22:55:32</t>
+    <t>18:43:52</t>
+  </si>
+  <si>
+    <t>20:20:23</t>
+  </si>
+  <si>
+    <t>21:57:20</t>
   </si>
   <si>
     <t>00:32:30</t>
@@ -355,19 +355,19 @@
     <t>19:35:43</t>
   </si>
   <si>
-    <t>21:12:19</t>
+    <t>21:12:20</t>
   </si>
   <si>
     <t>22:49:47</t>
   </si>
   <si>
-    <t>01:24:30</t>
-  </si>
-  <si>
-    <t>21:21:49</t>
-  </si>
-  <si>
-    <t>22:58:29</t>
+    <t>18:46:15</t>
+  </si>
+  <si>
+    <t>20:22:37</t>
+  </si>
+  <si>
+    <t>21:59:48</t>
   </si>
   <si>
     <t>00:35:16</t>
@@ -388,10 +388,10 @@
     <t>21:19:50</t>
   </si>
   <si>
-    <t>22:56:37</t>
-  </si>
-  <si>
-    <t>00:33:17</t>
+    <t>22:56:36</t>
+  </si>
+  <si>
+    <t>00:33:16</t>
   </si>
   <si>
     <t>20:30:26</t>
@@ -400,7 +400,7 @@
     <t>22:07:10</t>
   </si>
   <si>
-    <t>23:43:54</t>
+    <t>23:43:53</t>
   </si>
   <si>
     <t>19:40:59</t>
@@ -415,7 +415,7 @@
     <t>18:51:31</t>
   </si>
   <si>
-    <t>20:28:06</t>
+    <t>20:28:07</t>
   </si>
   <si>
     <t>22:04:53</t>
@@ -430,22 +430,22 @@
     <t>21:15:16</t>
   </si>
   <si>
-    <t>22:51:54</t>
-  </si>
-  <si>
-    <t>01:27:05</t>
-  </si>
-  <si>
-    <t>21:24:02</t>
-  </si>
-  <si>
-    <t>23:01:27</t>
+    <t>22:51:55</t>
+  </si>
+  <si>
+    <t>18:48:52</t>
+  </si>
+  <si>
+    <t>20:25:35</t>
+  </si>
+  <si>
+    <t>22:02:17</t>
   </si>
   <si>
     <t>00:38:03</t>
   </si>
   <si>
-    <t>20:34:16</t>
+    <t>20:34:15</t>
   </si>
   <si>
     <t>22:12:05</t>
@@ -499,19 +499,19 @@
     <t>19:41:18</t>
   </si>
   <si>
-    <t>21:18:12</t>
+    <t>21:18:13</t>
   </si>
   <si>
     <t>22:54:02</t>
   </si>
   <si>
-    <t>01:29:30</t>
-  </si>
-  <si>
-    <t>21:26:38</t>
-  </si>
-  <si>
-    <t>23:03:42</t>
+    <t>18:51:28</t>
+  </si>
+  <si>
+    <t>20:28:33</t>
+  </si>
+  <si>
+    <t>22:04:46</t>
   </si>
   <si>
     <t>00:40:23</t>
@@ -520,13 +520,13 @@
     <t>20:37:11</t>
   </si>
   <si>
-    <t>22:14:22</t>
+    <t>22:14:21</t>
   </si>
   <si>
     <t>23:51:09</t>
   </si>
   <si>
-    <t>01:27:10</t>
+    <t>01:27:09</t>
   </si>
   <si>
     <t>21:24:56</t>
@@ -562,16 +562,22 @@
     <t>22:10:02</t>
   </si>
   <si>
-    <t>23:45:58</t>
-  </si>
-  <si>
     <t>19:43:37</t>
   </si>
   <si>
     <t>21:20:27</t>
   </si>
   <si>
-    <t>22:56:40</t>
+    <t>22:56:41</t>
+  </si>
+  <si>
+    <t>18:53:52</t>
+  </si>
+  <si>
+    <t>20:30:47</t>
+  </si>
+  <si>
+    <t>22:07:14</t>
   </si>
   <si>
     <t>0°</t>
@@ -598,7 +604,7 @@
     <t>5°</t>
   </si>
   <si>
-    <t>01:29:39</t>
+    <t>18°</t>
   </si>
   <si>
     <t>20:26:32</t>
@@ -619,7 +625,13 @@
     <t>19:38:24</t>
   </si>
   <si>
-    <t>21:11:14</t>
+    <t>21:11:15</t>
+  </si>
+  <si>
+    <t>18:50:56</t>
+  </si>
+  <si>
+    <t>20:23:46</t>
   </si>
   <si>
     <t>B</t>
@@ -668,7 +680,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="24">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -683,7 +695,73 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF6AD26A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF558CC8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6697CD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF0707F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF77A3D3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC4D7EC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90B4DB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4E2F1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5E92CB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF3F9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF80A9D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -695,43 +773,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEF3F9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF88AED8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF0B070"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF80A9D6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF558CC8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF77A3D3"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6AD26A"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -743,25 +785,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF90B4DB"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6697CD"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFBBD1E9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6E9DD0"/>
+        <fgColor rgb="FFCCDCEE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -774,36 +804,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDE8F4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE6EEF7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD4E2F1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCDCEE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB2CBE6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -844,7 +844,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -916,12 +916,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1403,55 +1397,55 @@
         <v>18</v>
       </c>
       <c r="B2" s="2">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>194</v>
+        <v>70</v>
       </c>
       <c r="L2" s="4">
-        <v>-20.7</v>
+        <v>-25</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="O2" s="6">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="P2" s="7">
-        <v>44</v>
-      </c>
-      <c r="Q2" s="8">
-        <v>91</v>
-      </c>
-      <c r="R2" s="9">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="7">
+        <v>0</v>
+      </c>
+      <c r="R2" s="7">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -1459,54 +1453,54 @@
         <v>19</v>
       </c>
       <c r="B3" s="2">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L3" s="4">
-        <v>-23.7</v>
+        <v>-19.6</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O3" s="10">
-        <v>26</v>
-      </c>
-      <c r="P3" s="11">
-        <v>25</v>
-      </c>
-      <c r="Q3" s="12">
-        <v>1</v>
-      </c>
-      <c r="R3" s="12">
+        <v>209</v>
+      </c>
+      <c r="O3" s="6">
+        <v>0</v>
+      </c>
+      <c r="P3" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="7">
+        <v>0</v>
+      </c>
+      <c r="R3" s="7">
         <v>0</v>
       </c>
     </row>
@@ -1515,54 +1509,54 @@
         <v>20</v>
       </c>
       <c r="B4" s="2">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>44</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="L4" s="4">
-        <v>-27.8</v>
+        <v>-26.9</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O4" s="10">
-        <v>30</v>
-      </c>
-      <c r="P4" s="11">
-        <v>26</v>
-      </c>
-      <c r="Q4" s="12">
-        <v>0</v>
-      </c>
-      <c r="R4" s="12">
+        <v>208</v>
+      </c>
+      <c r="O4" s="6">
+        <v>1</v>
+      </c>
+      <c r="P4" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="7">
+        <v>1</v>
+      </c>
+      <c r="R4" s="7">
         <v>0</v>
       </c>
     </row>
@@ -1571,54 +1565,54 @@
         <v>21</v>
       </c>
       <c r="B5" s="2">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="L5" s="4">
-        <v>-25</v>
+        <v>-27.6</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O5" s="10">
-        <v>24</v>
-      </c>
-      <c r="P5" s="13">
-        <v>21</v>
-      </c>
-      <c r="Q5" s="12">
-        <v>0</v>
-      </c>
-      <c r="R5" s="12">
+        <v>208</v>
+      </c>
+      <c r="O5" s="6">
+        <v>1</v>
+      </c>
+      <c r="P5" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="7">
+        <v>1</v>
+      </c>
+      <c r="R5" s="7">
         <v>0</v>
       </c>
     </row>
@@ -1630,51 +1624,51 @@
         <v>13</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="L6" s="4">
-        <v>-19.6</v>
+        <v>-21.5</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="O6" s="14">
-        <v>0</v>
-      </c>
-      <c r="P6" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="12">
-        <v>0</v>
-      </c>
-      <c r="R6" s="12">
+        <v>209</v>
+      </c>
+      <c r="O6" s="6">
+        <v>11</v>
+      </c>
+      <c r="P6" s="8">
+        <v>11</v>
+      </c>
+      <c r="Q6" s="7">
+        <v>0</v>
+      </c>
+      <c r="R6" s="7">
         <v>0</v>
       </c>
     </row>
@@ -1683,54 +1677,54 @@
         <v>23</v>
       </c>
       <c r="B7" s="2">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="L7" s="4">
-        <v>-26.9</v>
+        <v>-24.2</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O7" s="14">
-        <v>0</v>
-      </c>
-      <c r="P7" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="12">
-        <v>0</v>
-      </c>
-      <c r="R7" s="12">
+        <v>208</v>
+      </c>
+      <c r="O7" s="6">
+        <v>0</v>
+      </c>
+      <c r="P7" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="7">
+        <v>0</v>
+      </c>
+      <c r="R7" s="7">
         <v>0</v>
       </c>
     </row>
@@ -1739,55 +1733,55 @@
         <v>24</v>
       </c>
       <c r="B8" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="L8" s="4">
-        <v>-27.6</v>
+        <v>-28.5</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O8" s="10">
-        <v>48</v>
-      </c>
-      <c r="P8" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="15">
-        <v>41</v>
-      </c>
-      <c r="R8" s="15">
-        <v>41</v>
+        <v>208</v>
+      </c>
+      <c r="O8" s="6">
+        <v>0</v>
+      </c>
+      <c r="P8" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="7">
+        <v>0</v>
+      </c>
+      <c r="R8" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -1795,55 +1789,55 @@
         <v>25</v>
       </c>
       <c r="B9" s="2">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="L9" s="4">
-        <v>-21.5</v>
+        <v>-25.7</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="O9" s="6">
-        <v>49</v>
-      </c>
-      <c r="P9" s="12">
-        <v>2</v>
-      </c>
-      <c r="Q9" s="16">
-        <v>36</v>
-      </c>
-      <c r="R9" s="17">
-        <v>9</v>
+        <v>0</v>
+      </c>
+      <c r="P9" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="7">
+        <v>0</v>
+      </c>
+      <c r="R9" s="7">
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -1851,55 +1845,55 @@
         <v>26</v>
       </c>
       <c r="B10" s="2">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>75</v>
+        <v>197</v>
       </c>
       <c r="L10" s="4">
-        <v>-24.2</v>
+        <v>-20</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O10" s="14">
-        <v>0</v>
-      </c>
-      <c r="P10" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="12">
-        <v>0</v>
-      </c>
-      <c r="R10" s="12">
-        <v>0</v>
+        <v>208</v>
+      </c>
+      <c r="O10" s="9">
+        <v>63</v>
+      </c>
+      <c r="P10" s="10">
+        <v>18</v>
+      </c>
+      <c r="Q10" s="10">
+        <v>19</v>
+      </c>
+      <c r="R10" s="11">
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -1910,52 +1904,52 @@
         <v>30</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="L11" s="4">
-        <v>-28.5</v>
+        <v>-27.5</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O11" s="14">
-        <v>0</v>
-      </c>
-      <c r="P11" s="12">
-        <v>0</v>
+        <v>208</v>
+      </c>
+      <c r="O11" s="9">
+        <v>81</v>
+      </c>
+      <c r="P11" s="8">
+        <v>8</v>
       </c>
       <c r="Q11" s="12">
-        <v>0</v>
-      </c>
-      <c r="R11" s="12">
-        <v>0</v>
+        <v>33</v>
+      </c>
+      <c r="R11" s="13">
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -1963,55 +1957,55 @@
         <v>28</v>
       </c>
       <c r="B12" s="2">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>173</v>
+        <v>145</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="L12" s="4">
-        <v>-25.7</v>
+        <v>-28.3</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O12" s="14">
-        <v>0</v>
-      </c>
-      <c r="P12" s="12">
-        <v>0</v>
+        <v>208</v>
+      </c>
+      <c r="O12" s="9">
+        <v>97</v>
+      </c>
+      <c r="P12" s="14">
+        <v>6</v>
       </c>
       <c r="Q12" s="12">
-        <v>0</v>
-      </c>
-      <c r="R12" s="12">
-        <v>0</v>
+        <v>35</v>
+      </c>
+      <c r="R12" s="15">
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -2019,55 +2013,55 @@
         <v>29</v>
       </c>
       <c r="B13" s="2">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="L13" s="4">
-        <v>-20</v>
+        <v>-14.7</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O13" s="6">
-        <v>95</v>
-      </c>
-      <c r="P13" s="13">
-        <v>20</v>
-      </c>
-      <c r="Q13" s="12">
-        <v>0</v>
-      </c>
-      <c r="R13" s="8">
-        <v>88</v>
+        <v>210</v>
+      </c>
+      <c r="O13" s="9">
+        <v>100</v>
+      </c>
+      <c r="P13" s="8">
+        <v>10</v>
+      </c>
+      <c r="Q13" s="10">
+        <v>19</v>
+      </c>
+      <c r="R13" s="16">
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -2078,52 +2072,52 @@
         <v>30</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>79</v>
+        <v>199</v>
       </c>
       <c r="L14" s="4">
-        <v>-27.5</v>
+        <v>-24.7</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O14" s="6">
-        <v>84</v>
-      </c>
-      <c r="P14" s="13">
-        <v>18</v>
-      </c>
-      <c r="Q14" s="11">
-        <v>26</v>
+        <v>208</v>
+      </c>
+      <c r="O14" s="9">
+        <v>78</v>
+      </c>
+      <c r="P14" s="8">
+        <v>9</v>
+      </c>
+      <c r="Q14" s="17">
+        <v>23</v>
       </c>
       <c r="R14" s="18">
-        <v>61</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -2131,55 +2125,55 @@
         <v>31</v>
       </c>
       <c r="B15" s="2">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>52</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>145</v>
+        <v>178</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="L15" s="4">
-        <v>-28.3</v>
+        <v>-29.2</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O15" s="6">
-        <v>73</v>
-      </c>
-      <c r="P15" s="19">
-        <v>13</v>
-      </c>
-      <c r="Q15" s="11">
-        <v>26</v>
-      </c>
-      <c r="R15" s="20">
-        <v>50</v>
+        <v>208</v>
+      </c>
+      <c r="O15" s="9">
+        <v>70</v>
+      </c>
+      <c r="P15" s="8">
+        <v>8</v>
+      </c>
+      <c r="Q15" s="17">
+        <v>24</v>
+      </c>
+      <c r="R15" s="19">
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -2187,55 +2181,55 @@
         <v>32</v>
       </c>
       <c r="B16" s="2">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="L16" s="4">
-        <v>-14.6</v>
+        <v>-8.4</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="O16" s="6">
-        <v>90</v>
-      </c>
-      <c r="P16" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="13">
-        <v>18</v>
-      </c>
-      <c r="R16" s="21">
-        <v>79</v>
+        <v>209</v>
+      </c>
+      <c r="O16" s="9">
+        <v>100</v>
+      </c>
+      <c r="P16" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="20">
+        <v>42</v>
+      </c>
+      <c r="R16" s="16">
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -2243,55 +2237,55 @@
         <v>33</v>
       </c>
       <c r="B17" s="2">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="L17" s="4">
-        <v>-24.7</v>
+        <v>-20.4</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O17" s="6">
-        <v>92</v>
-      </c>
-      <c r="P17" s="19">
-        <v>17</v>
-      </c>
-      <c r="Q17" s="15">
-        <v>41</v>
-      </c>
-      <c r="R17" s="22">
-        <v>84</v>
+        <v>210</v>
+      </c>
+      <c r="O17" s="9">
+        <v>71</v>
+      </c>
+      <c r="P17" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="21">
+        <v>59</v>
+      </c>
+      <c r="R17" s="12">
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -2299,55 +2293,55 @@
         <v>34</v>
       </c>
       <c r="B18" s="2">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="L18" s="4">
-        <v>-29.2</v>
+        <v>-28.1</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O18" s="6">
-        <v>89</v>
-      </c>
-      <c r="P18" s="19">
-        <v>13</v>
-      </c>
-      <c r="Q18" s="7">
-        <v>46</v>
-      </c>
-      <c r="R18" s="23">
-        <v>76</v>
+        <v>208</v>
+      </c>
+      <c r="O18" s="9">
+        <v>66</v>
+      </c>
+      <c r="P18" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="12">
+        <v>34</v>
+      </c>
+      <c r="R18" s="18">
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -2355,55 +2349,55 @@
         <v>35</v>
       </c>
       <c r="B19" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>179</v>
+        <v>121</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>198</v>
+        <v>87</v>
       </c>
       <c r="L19" s="4">
-        <v>-8.4</v>
+        <v>-29.1</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="O19" s="6">
-        <v>99</v>
-      </c>
-      <c r="P19" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="21">
-        <v>79</v>
-      </c>
-      <c r="R19" s="18">
-        <v>60</v>
+        <v>209</v>
+      </c>
+      <c r="O19" s="9">
+        <v>77</v>
+      </c>
+      <c r="P19" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="17">
+        <v>24</v>
+      </c>
+      <c r="R19" s="11">
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:18">
@@ -2411,55 +2405,55 @@
         <v>36</v>
       </c>
       <c r="B20" s="2">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="L20" s="4">
-        <v>-20.4</v>
+        <v>-15</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="O20" s="6">
-        <v>100</v>
-      </c>
-      <c r="P20" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="24">
-        <v>68</v>
-      </c>
-      <c r="R20" s="22">
-        <v>86</v>
+        <v>210</v>
+      </c>
+      <c r="O20" s="9">
+        <v>79</v>
+      </c>
+      <c r="P20" s="22">
+        <v>70</v>
+      </c>
+      <c r="Q20" s="22">
+        <v>70</v>
+      </c>
+      <c r="R20" s="21">
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:18">
@@ -2467,55 +2461,55 @@
         <v>37</v>
       </c>
       <c r="B21" s="2">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="L21" s="4">
+        <v>-25.2</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="O21" s="9">
         <v>57</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="L21" s="4">
-        <v>-28.1</v>
-      </c>
-      <c r="M21" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O21" s="6">
-        <v>99</v>
-      </c>
-      <c r="P21" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="7">
-        <v>47</v>
-      </c>
-      <c r="R21" s="25">
-        <v>98</v>
+      <c r="P21" s="23">
+        <v>48</v>
+      </c>
+      <c r="Q21" s="17">
+        <v>23</v>
+      </c>
+      <c r="R21" s="12">
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:18">
@@ -2523,55 +2517,55 @@
         <v>38</v>
       </c>
       <c r="B22" s="2">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="L22" s="4">
-        <v>-29.1</v>
+        <v>-29.8</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="O22" s="6">
-        <v>100</v>
-      </c>
-      <c r="P22" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="26">
-        <v>54</v>
-      </c>
-      <c r="R22" s="25">
-        <v>99</v>
+        <v>208</v>
+      </c>
+      <c r="O22" s="9">
+        <v>45</v>
+      </c>
+      <c r="P22" s="19">
+        <v>28</v>
+      </c>
+      <c r="Q22" s="7">
+        <v>0</v>
+      </c>
+      <c r="R22" s="14">
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:18">
@@ -2579,55 +2573,55 @@
         <v>39</v>
       </c>
       <c r="B23" s="2">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="L23" s="4">
-        <v>-15</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="O23" s="6">
-        <v>85</v>
-      </c>
-      <c r="P23" s="9">
-        <v>29</v>
-      </c>
-      <c r="Q23" s="18">
-        <v>60</v>
-      </c>
-      <c r="R23" s="17">
-        <v>9</v>
+        <v>210</v>
+      </c>
+      <c r="O23" s="9">
+        <v>76</v>
+      </c>
+      <c r="P23" s="12">
+        <v>37</v>
+      </c>
+      <c r="Q23" s="19">
+        <v>30</v>
+      </c>
+      <c r="R23" s="18">
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:18">
@@ -2635,55 +2629,55 @@
         <v>40</v>
       </c>
       <c r="B24" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="L24" s="4">
+        <v>-20.9</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="O24" s="9">
+        <v>74</v>
+      </c>
+      <c r="P24" s="8">
+        <v>9</v>
+      </c>
+      <c r="Q24" s="20">
+        <v>41</v>
+      </c>
+      <c r="R24" s="21">
         <v>62</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="K24" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="L24" s="4">
-        <v>-25.2</v>
-      </c>
-      <c r="M24" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="N24" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O24" s="6">
-        <v>59</v>
-      </c>
-      <c r="P24" s="19">
-        <v>17</v>
-      </c>
-      <c r="Q24" s="9">
-        <v>28</v>
-      </c>
-      <c r="R24" s="13">
-        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:18">
@@ -2691,55 +2685,55 @@
         <v>41</v>
       </c>
       <c r="B25" s="2">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="L25" s="4">
-        <v>-29.8</v>
+        <v>-28.7</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O25" s="10">
-        <v>45</v>
-      </c>
-      <c r="P25" s="17">
-        <v>9</v>
-      </c>
-      <c r="Q25" s="17">
-        <v>11</v>
-      </c>
-      <c r="R25" s="13">
-        <v>22</v>
+        <v>208</v>
+      </c>
+      <c r="O25" s="9">
+        <v>94</v>
+      </c>
+      <c r="P25" s="14">
+        <v>5</v>
+      </c>
+      <c r="Q25" s="24">
+        <v>78</v>
+      </c>
+      <c r="R25" s="15">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>